<commit_message>
Add equipment data to the drawer
</commit_message>
<xml_diff>
--- a/data/raw/rules/rules.xlsx
+++ b/data/raw/rules/rules.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="180">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -434,6 +434,132 @@
   </si>
   <si>
     <t xml:space="preserve">woodland-creature</t>
+  </si>
+  <si>
+    <t xml:space="preserve">barge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">brutal-power-attack</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 90)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hurl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 91)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hand-weapon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">equipment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 103)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">two-handed-weapon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hand-and-a-half-weapon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">unarmed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">spear</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 104)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pike</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 105)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">war-spear</t>
+  </si>
+  <si>
+    <t xml:space="preserve">whip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">elven-weapon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">master-forged</t>
+  </si>
+  <si>
+    <t xml:space="preserve">staff-of-power</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 106)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">throwing-weapon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">crossbow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">blowpipe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">banner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 107)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">elven-cloak</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 108)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">war-drum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">war-horn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">armour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 109)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">light-armour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">heavy-armour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">heavy-dwarf-armour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mithril-armour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">shield</t>
+  </si>
+  <si>
+    <t xml:space="preserve">light-shield</t>
   </si>
 </sst>
 </file>
@@ -443,7 +569,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
@@ -465,12 +591,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -515,7 +635,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -530,10 +650,6 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -553,12 +669,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D102"/>
-  <sheetFormatPr defaultColWidth="8.50390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:D134"/>
+  <sheetFormatPr defaultColWidth="8.51171875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13.41"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="23.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.95"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="9.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="53.45"/>
   </cols>
   <sheetData>
@@ -1502,7 +1618,7 @@
       <c r="C68" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="D68" s="4" t="s">
+      <c r="D68" s="2" t="s">
         <v>95</v>
       </c>
     </row>
@@ -1684,7 +1800,7 @@
       <c r="C81" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="D81" s="4" t="s">
+      <c r="D81" s="2" t="s">
         <v>95</v>
       </c>
     </row>
@@ -1712,7 +1828,7 @@
       <c r="C83" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="D83" s="4" t="s">
+      <c r="D83" s="2" t="s">
         <v>95</v>
       </c>
     </row>
@@ -1778,7 +1894,7 @@
       <c r="C88" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="D88" s="4" t="s">
+      <c r="D88" s="2" t="s">
         <v>95</v>
       </c>
     </row>
@@ -1916,7 +2032,7 @@
       <c r="C98" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="D98" s="4" t="s">
+      <c r="D98" s="2" t="s">
         <v>95</v>
       </c>
     </row>
@@ -1975,6 +2091,350 @@
       <c r="D102" s="2" t="s">
         <v>135</v>
       </c>
+    </row>
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="0" t="s">
+        <v>138</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="D103" s="2" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="0" t="s">
+        <v>141</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="D104" s="2" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="0" t="s">
+        <v>142</v>
+      </c>
+      <c r="B105" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="D105" s="2" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="0" t="s">
+        <v>144</v>
+      </c>
+      <c r="B106" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D106" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="0" t="s">
+        <v>147</v>
+      </c>
+      <c r="B107" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D107" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="0" t="s">
+        <v>148</v>
+      </c>
+      <c r="B108" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D108" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="0" t="s">
+        <v>149</v>
+      </c>
+      <c r="B109" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D109" s="2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="0" t="s">
+        <v>150</v>
+      </c>
+      <c r="B110" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D110" s="2" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="B111" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D111" s="2" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="0" t="s">
+        <v>153</v>
+      </c>
+      <c r="B112" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D112" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="0" t="s">
+        <v>155</v>
+      </c>
+      <c r="B113" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D113" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="0" t="s">
+        <v>156</v>
+      </c>
+      <c r="B114" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D114" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="0" t="s">
+        <v>157</v>
+      </c>
+      <c r="B115" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D115" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="0" t="s">
+        <v>158</v>
+      </c>
+      <c r="B116" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D116" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="0" t="s">
+        <v>159</v>
+      </c>
+      <c r="B117" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D117" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A118" s="0" t="s">
+        <v>160</v>
+      </c>
+      <c r="B118" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D118" s="2" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A119" s="0" t="s">
+        <v>162</v>
+      </c>
+      <c r="B119" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D119" s="2" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A120" s="0" t="s">
+        <v>163</v>
+      </c>
+      <c r="B120" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D120" s="2" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A121" s="0" t="s">
+        <v>164</v>
+      </c>
+      <c r="B121" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D121" s="2" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A122" s="0" t="s">
+        <v>165</v>
+      </c>
+      <c r="B122" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D122" s="2" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A123" s="0" t="s">
+        <v>166</v>
+      </c>
+      <c r="B123" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D123" s="2" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A124" s="0" t="s">
+        <v>168</v>
+      </c>
+      <c r="B124" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D124" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A125" s="0" t="s">
+        <v>170</v>
+      </c>
+      <c r="B125" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D125" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A126" s="0" t="s">
+        <v>171</v>
+      </c>
+      <c r="B126" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D126" s="2" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A127" s="0" t="s">
+        <v>172</v>
+      </c>
+      <c r="B127" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D127" s="2" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A128" s="0" t="s">
+        <v>174</v>
+      </c>
+      <c r="B128" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D128" s="2" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A129" s="0" t="s">
+        <v>175</v>
+      </c>
+      <c r="B129" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D129" s="2" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A130" s="0" t="s">
+        <v>176</v>
+      </c>
+      <c r="B130" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D130" s="2" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A131" s="0" t="s">
+        <v>177</v>
+      </c>
+      <c r="B131" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D131" s="2" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A132" s="0" t="s">
+        <v>178</v>
+      </c>
+      <c r="B132" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D132" s="2" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A133" s="0" t="s">
+        <v>179</v>
+      </c>
+      <c r="B133" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D133" s="2" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D134" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Amend rule texts with keyword and errata markers
</commit_message>
<xml_diff>
--- a/data/raw/rules/rules.xlsx
+++ b/data/raw/rules/rules.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="457" uniqueCount="166">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -241,12 +241,6 @@
     <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 124)</t>
   </si>
   <si>
-    <t xml:space="preserve">arcing-shot</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 141)</t>
-  </si>
-  <si>
     <t xml:space="preserve">backstabbers</t>
   </si>
   <si>
@@ -274,9 +268,6 @@
     <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 125)</t>
   </si>
   <si>
-    <t xml:space="preserve">direct-shot</t>
-  </si>
-  <si>
     <t xml:space="preserve">dominant</t>
   </si>
   <si>
@@ -295,27 +286,15 @@
     <t xml:space="preserve">fell-sight</t>
   </si>
   <si>
-    <t xml:space="preserve">flaming-ammunition</t>
-  </si>
-  <si>
     <t xml:space="preserve">fly</t>
   </si>
   <si>
     <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 126)</t>
   </si>
   <si>
-    <t xml:space="preserve">foul-temperament</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Armies of The Lord of The Rings™(page 193)</t>
-  </si>
-  <si>
     <t xml:space="preserve">general-hunter</t>
   </si>
   <si>
-    <t xml:space="preserve">gnarled-hide</t>
-  </si>
-  <si>
     <t xml:space="preserve">harbinger-of-evil</t>
   </si>
   <si>
@@ -358,21 +337,12 @@
     <t xml:space="preserve">poisoned-attacks</t>
   </si>
   <si>
-    <t xml:space="preserve">rappelling-lines</t>
-  </si>
-  <si>
     <t xml:space="preserve">resistant-to-magic</t>
   </si>
   <si>
-    <t xml:space="preserve">rocks</t>
-  </si>
-  <si>
     <t xml:space="preserve">set-ablaze</t>
   </si>
   <si>
-    <t xml:space="preserve">severed-heads</t>
-  </si>
-  <si>
     <t xml:space="preserve">sharpshooter</t>
   </si>
   <si>
@@ -382,21 +352,12 @@
     <t xml:space="preserve">shieldwall</t>
   </si>
   <si>
-    <t xml:space="preserve">sigils-of-defiance</t>
-  </si>
-  <si>
     <t xml:space="preserve">spectral-walk</t>
   </si>
   <si>
     <t xml:space="preserve">stalk-unseen</t>
   </si>
   <si>
-    <t xml:space="preserve">static</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Middle-earth™ Strategy Battle Game Rules Manual (page 140)</t>
-  </si>
-  <si>
     <t xml:space="preserve">survival-instinct</t>
   </si>
   <si>
@@ -416,9 +377,6 @@
   </si>
   <si>
     <t xml:space="preserve">timid</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tusk-weapons</t>
   </si>
   <si>
     <t xml:space="preserve">unyielding-combat-stance</t>
@@ -669,8 +627,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D134"/>
-  <sheetFormatPr defaultColWidth="8.51171875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:D123"/>
+  <sheetFormatPr defaultColWidth="8.51953125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="23.6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.95"/>
@@ -1357,14 +1315,16 @@
       <c r="B49" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="C49" s="3"/>
+      <c r="C49" s="3" t="s">
+        <v>71</v>
+      </c>
       <c r="D49" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B50" s="3" t="s">
         <v>70</v>
@@ -1378,7 +1338,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B51" s="3" t="s">
         <v>70</v>
@@ -1392,7 +1352,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B52" s="3" t="s">
         <v>70</v>
@@ -1406,13 +1366,13 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C53" s="3" t="s">
         <v>78</v>
-      </c>
-      <c r="B53" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C53" s="3" t="s">
-        <v>71</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>72</v>
@@ -1426,7 +1386,7 @@
         <v>70</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D54" s="2" t="s">
         <v>72</v>
@@ -1434,16 +1394,16 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C55" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="D55" s="2" t="s">
         <v>81</v>
-      </c>
-      <c r="B55" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C55" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="D55" s="2" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1454,92 +1414,94 @@
         <v>70</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B57" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="C57" s="3"/>
+      <c r="C57" s="3" t="s">
+        <v>71</v>
+      </c>
       <c r="D57" s="2" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B58" s="3" t="s">
         <v>70</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B59" s="3" t="s">
         <v>70</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B60" s="3" t="s">
         <v>70</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B61" s="3" t="s">
         <v>70</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C62" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="D62" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="B62" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C62" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="D62" s="2" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1550,10 +1512,10 @@
         <v>70</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1563,8 +1525,12 @@
       <c r="B64" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="C64" s="3"/>
-      <c r="D64" s="2"/>
+      <c r="C64" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="2" t="s">
@@ -1577,68 +1543,68 @@
         <v>71</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C66" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="D66" s="2" t="s">
         <v>94</v>
-      </c>
-      <c r="B66" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C66" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="D66" s="2" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B67" s="3" t="s">
         <v>70</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B68" s="3" t="s">
         <v>70</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B69" s="3" t="s">
         <v>70</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B70" s="3" t="s">
         <v>70</v>
@@ -1647,32 +1613,32 @@
         <v>71</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B71" s="3" t="s">
         <v>70</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="2" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B72" s="3" t="s">
         <v>70</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D72" s="2" t="s">
         <v>101</v>
@@ -1680,13 +1646,13 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B73" s="3" t="s">
         <v>70</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="D73" s="2" t="s">
         <v>101</v>
@@ -1694,13 +1660,13 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B74" s="3" t="s">
         <v>70</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="D74" s="2" t="s">
         <v>101</v>
@@ -1708,7 +1674,7 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B75" s="3" t="s">
         <v>70</v>
@@ -1722,13 +1688,13 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B76" s="3" t="s">
         <v>70</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="D76" s="2" t="s">
         <v>101</v>
@@ -1736,21 +1702,21 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B77" s="3" t="s">
         <v>70</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B78" s="3" t="s">
         <v>70</v>
@@ -1764,7 +1730,7 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B79" s="3" t="s">
         <v>70</v>
@@ -1778,13 +1744,13 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B80" s="3" t="s">
         <v>70</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="D80" s="2" t="s">
         <v>108</v>
@@ -1792,27 +1758,27 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B81" s="3" t="s">
         <v>70</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B82" s="3" t="s">
         <v>70</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="D82" s="2" t="s">
         <v>108</v>
@@ -1820,7 +1786,7 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B83" s="3" t="s">
         <v>70</v>
@@ -1829,21 +1795,21 @@
         <v>71</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B84" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C84" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="D84" s="2" t="s">
         <v>115</v>
-      </c>
-      <c r="B84" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C84" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="D84" s="2" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1853,8 +1819,12 @@
       <c r="B85" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="C85" s="3"/>
-      <c r="D85" s="2"/>
+      <c r="C85" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="D85" s="2" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="2" t="s">
@@ -1867,49 +1837,49 @@
         <v>71</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B87" s="3" t="s">
         <v>70</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B88" s="3" t="s">
         <v>70</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>95</v>
+        <v>115</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B89" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C89" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="D89" s="2" t="s">
         <v>121</v>
-      </c>
-      <c r="B89" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C89" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="D89" s="2" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1920,10 +1890,10 @@
         <v>70</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1933,171 +1903,140 @@
       <c r="B91" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="C91" s="3"/>
+      <c r="C91" s="3" t="s">
+        <v>71</v>
+      </c>
       <c r="D91" s="2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="0" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="2" t="s">
+      <c r="B92" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="B92" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C92" s="3" t="s">
-        <v>71</v>
-      </c>
       <c r="D92" s="2" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="2" t="s">
+      <c r="A93" s="0" t="s">
+        <v>127</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="D93" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="B93" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C93" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D93" s="2" t="s">
-        <v>118</v>
-      </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="B94" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C94" s="3" t="s">
-        <v>80</v>
+      <c r="A94" s="0" t="s">
+        <v>128</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>125</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="B95" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C95" s="3" t="s">
-        <v>80</v>
+      <c r="A95" s="0" t="s">
+        <v>130</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>131</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="B96" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C96" s="3" t="s">
-        <v>71</v>
+      <c r="A96" s="0" t="s">
+        <v>133</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>131</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="B97" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C97" s="3" t="s">
-        <v>80</v>
+      <c r="A97" s="0" t="s">
+        <v>134</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>131</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="2" t="s">
+      <c r="A98" s="0" t="s">
+        <v>135</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="D98" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="B98" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C98" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D98" s="2" t="s">
-        <v>95</v>
-      </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A99" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="B99" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C99" s="3" t="s">
-        <v>71</v>
+      <c r="A99" s="0" t="s">
+        <v>136</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>131</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>128</v>
+        <v>137</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="B100" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C100" s="3" t="s">
-        <v>71</v>
+      <c r="A100" s="0" t="s">
+        <v>138</v>
+      </c>
+      <c r="B100" s="1" t="s">
+        <v>131</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="B101" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C101" s="3" t="s">
-        <v>80</v>
+      <c r="A101" s="0" t="s">
+        <v>139</v>
+      </c>
+      <c r="B101" s="1" t="s">
+        <v>131</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A102" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="B102" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="C102" s="3" t="s">
-        <v>71</v>
+      <c r="A102" s="0" t="s">
+        <v>141</v>
+      </c>
+      <c r="B102" s="1" t="s">
+        <v>131</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="0" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="D103" s="2" t="s">
         <v>140</v>
@@ -2105,10 +2044,10 @@
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="0" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="D104" s="2" t="s">
         <v>140</v>
@@ -2116,35 +2055,35 @@
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="0" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="0" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>145</v>
+        <v>131</v>
       </c>
       <c r="D106" s="2" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="0" t="s">
+        <v>146</v>
+      </c>
+      <c r="B107" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="D107" s="2" t="s">
         <v>147</v>
-      </c>
-      <c r="B107" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="D107" s="2" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2152,10 +2091,10 @@
         <v>148</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>145</v>
+        <v>131</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2163,10 +2102,10 @@
         <v>149</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>145</v>
+        <v>131</v>
       </c>
       <c r="D109" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2174,43 +2113,43 @@
         <v>150</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>145</v>
+        <v>131</v>
       </c>
       <c r="D110" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="0" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>145</v>
+        <v>131</v>
       </c>
       <c r="D111" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="0" t="s">
+        <v>152</v>
+      </c>
+      <c r="B112" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="D112" s="2" t="s">
         <v>153</v>
-      </c>
-      <c r="B112" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="D112" s="2" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="0" t="s">
+        <v>154</v>
+      </c>
+      <c r="B113" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="D113" s="2" t="s">
         <v>155</v>
-      </c>
-      <c r="B113" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="D113" s="2" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2218,10 +2157,10 @@
         <v>156</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>145</v>
+        <v>131</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2229,10 +2168,10 @@
         <v>157</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>145</v>
+        <v>131</v>
       </c>
       <c r="D115" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2240,32 +2179,32 @@
         <v>158</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>145</v>
+        <v>131</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="0" t="s">
+        <v>160</v>
+      </c>
+      <c r="B117" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="D117" s="2" t="s">
         <v>159</v>
-      </c>
-      <c r="B117" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="D117" s="2" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="0" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>145</v>
+        <v>131</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2273,10 +2212,10 @@
         <v>162</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>145</v>
+        <v>131</v>
       </c>
       <c r="D119" s="2" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2284,10 +2223,10 @@
         <v>163</v>
       </c>
       <c r="B120" s="1" t="s">
-        <v>145</v>
+        <v>131</v>
       </c>
       <c r="D120" s="2" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2295,10 +2234,10 @@
         <v>164</v>
       </c>
       <c r="B121" s="1" t="s">
-        <v>145</v>
+        <v>131</v>
       </c>
       <c r="D121" s="2" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2306,135 +2245,14 @@
         <v>165</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>145</v>
+        <v>131</v>
       </c>
       <c r="D122" s="2" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A123" s="0" t="s">
-        <v>166</v>
-      </c>
-      <c r="B123" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="D123" s="2" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A124" s="0" t="s">
-        <v>168</v>
-      </c>
-      <c r="B124" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="D124" s="2" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A125" s="0" t="s">
-        <v>170</v>
-      </c>
-      <c r="B125" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="D125" s="2" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A126" s="0" t="s">
-        <v>171</v>
-      </c>
-      <c r="B126" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="D126" s="2" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A127" s="0" t="s">
-        <v>172</v>
-      </c>
-      <c r="B127" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="D127" s="2" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A128" s="0" t="s">
-        <v>174</v>
-      </c>
-      <c r="B128" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="D128" s="2" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A129" s="0" t="s">
-        <v>175</v>
-      </c>
-      <c r="B129" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="D129" s="2" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A130" s="0" t="s">
-        <v>176</v>
-      </c>
-      <c r="B130" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="D130" s="2" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A131" s="0" t="s">
-        <v>177</v>
-      </c>
-      <c r="B131" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="D131" s="2" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A132" s="0" t="s">
-        <v>178</v>
-      </c>
-      <c r="B132" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="D132" s="2" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A133" s="0" t="s">
-        <v>179</v>
-      </c>
-      <c r="B133" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="D133" s="2" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D134" s="2"/>
+      <c r="D123" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Migratie the old profiles into a new excel file
</commit_message>
<xml_diff>
--- a/data/raw/rules/rules.xlsx
+++ b/data/raw/rules/rules.xlsx
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="rules" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Rules" sheetId="1" state="visible" r:id="rId2"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -628,7 +628,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D123"/>
-  <sheetFormatPr defaultColWidth="8.51953125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5234375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="23.6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.95"/>

</xml_diff>